<commit_message>
26.10.28 LYJ: Gantry 관련 회의 커밋
</commit_message>
<xml_diff>
--- a/docu/공정비트.xlsx
+++ b/docu/공정비트.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EZEN\Desktop\LYJ\UNITY\project\docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44FA1987-102C-42BD-AE25-244CCEE9E0E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C76E83-8EB9-41B1-8B46-D27B08D14B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="8835" windowWidth="14610" windowHeight="6750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1차" sheetId="3" r:id="rId1"/>
@@ -1726,294 +1726,302 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>232</v>
       </c>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16" s="2">
         <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="2" t="s">
         <v>259</v>
       </c>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="2" t="s">
         <v>260</v>
       </c>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="2" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="2" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="2" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="2" t="s">
         <v>265</v>
       </c>
+      <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2602,147 +2610,164 @@
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="3" t="s">
+      <c r="A60" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
+      <c r="A61" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" s="2" t="s">
         <v>119</v>
       </c>
+      <c r="C61" s="2"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+      <c r="A62" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" s="2" t="s">
         <v>120</v>
       </c>
+      <c r="C62" s="2"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
+      <c r="A63" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="C63" s="2"/>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
+      <c r="A64" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
+      <c r="C64" s="2"/>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
+      <c r="C65" s="2"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" s="2" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
+      <c r="C66" s="2"/>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
+      <c r="C67" s="2"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
+      <c r="C69" s="2"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" s="2" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
+      <c r="C70" s="2"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
+      <c r="C71" s="2"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" s="2" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
+      <c r="C72" s="2"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="1" t="s">
+      <c r="C73" s="2"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="1" t="s">
+      <c r="C74" s="2"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
+      <c r="C75" s="2"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
+      <c r="C76" s="2"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" s="2" t="s">
         <v>169</v>
       </c>
+      <c r="C77" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>